<commit_message>
copy: new homepage and shared figures from the concise copy document
Batch 1 of the copy replacement (RTG_Website_Copy_Concise.docx, Draft 1).

Homepage rebuilt to the document's order, eleven sections down to seven:
hero and four figures, the family business with client names, engineered
for offshore conditions with the showroom, sectors, equipment rows, the
four-tier ladder, service life support. Fleet, Stats, ProofCase and
EquipmentGrid are gone, along with the case-study WebGL stage.

Shared: PROOF gains since (1978) and staff (80) and loses the 22-years
figure; the standard band is four figures on every page; footer
strapline replaced. H-01 title, description and h1 updated in the
workbook and regenerated.

Client names are published as written, decided by the site owner on
2026-10-08 and recorded in CLAUDE.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WYL1dwTrpuG7Wg2RUY2FW
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Deck Equipment for Research &amp; Survey Vessels | RTG</t>
+          <t>Deck Machinery for Research, Survey &amp; Offshore Vessels | RTG</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -617,7 +617,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Custom winches, launch and recovery systems and deck machinery for research, survey and geotechnical vessels. Designed in the UK, built and tested in the EU.</t>
+          <t>Custom winches, LARS, tensioners and cranes for research, survey and offshore vessels. Family business since 1978. Designed in the UK, built and tested in the EU.</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Deck equipment built for the work, not the brochure</t>
+          <t>Custom deck machinery for research, survey and offshore vessels</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">

</xml_diff>

<commit_message>
copy: sector pages from the concise copy document
Batch 2 of the copy replacement. S-00 to S-07 rewritten as short headed
lists; the Sector template drops the tall picture column, the
technical-note sequence and the featured-case band, and sets the lists in
two columns. Related equipment now points at the right product pages.

A page's closing block may be just its buttons, taken from the hero, and
the standard band now sits directly above the footer.

Titles, descriptions and h1s updated in the workbook. The S-00 title was
shortened from 78 characters to fit the 60-character audit limit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WYL1dwTrpuG7Wg2RUY2FW
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Sectors We Supply | Survey, Geotechnical, Wind | RTG</t>
+          <t>Sectors | Survey, Geotechnical, Wind, Seismic, Subsea | RTG</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -723,7 +723,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>RTG deck equipment works across ocean survey, marine geotechnical, offshore wind and cables, seismic, research, subsea and defence. Find your sector.</t>
+          <t>RTG deck machinery for ocean survey, marine geotechnical, offshore wind and cables, seismic, oceanographic research, subsea and defence vessels.</t>
         </is>
       </c>
       <c r="L3" t="n">
@@ -731,7 +731,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>The sectors we build for</t>
+          <t>Deck handling systems for seven offshore sectors</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Winches and launch and recovery systems for hydrographic and geophysical survey: CTD, side scan, magnetometer, sub-bottom profiler and deep tow, 300 to 4,000 m.</t>
+          <t>Winches and LARS for hydrographic and geophysical survey: CTD, side scan, magnetometer, sub-bottom profiler and deep tow, 300 to 4,000 m.</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -837,7 +837,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Handling systems for survey and hydrographic work</t>
+          <t>Survey and hydrographic handling systems</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Corer, CPT and vibrocorer handling systems with tension control for seabed sampling. Proven to a 3,000 m working depth on a CPT sampling system.</t>
+          <t>Corer, CPT and vibrocorer handling systems with constant tension control for seabed sampling. Proven to 3,000 m working depth on a CPT sampling system.</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -943,7 +943,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>When the tool is fixed to the seabed and the ship is not</t>
+          <t>Geotechnical handling systems, proven to 3,000 m</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Site investigation handling, cable tensioners from 5 to 20 tonnes and containerised cable spreads for offshore wind arrays, export cables and interconnectors.</t>
+          <t>Site-investigation handling, 5 to 20 tonne cable tensioners and containerised cable spreads for offshore wind arrays, export cables and interconnectors.</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Every turbine starts with a core sample. Every array ends with a cable.</t>
+          <t>Site investigation and cable handling for offshore wind</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Seismic winches, source handling and streamer deployment systems for 2D and 3D marine seismic acquisition, designed for continuous duty at sea.</t>
+          <t>Seismic winches, source handling and streamer deployment systems for 2D and 3D marine seismic acquisition, designed for continuous duty.</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Seismic handling built for continuous duty</t>
+          <t>Seismic handling for continuous duty</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Research winches for CTD, coring and deep tow work, from 300 to 4,000 m, electric or hydraulic, with precise slow-speed control for repeatable casts.</t>
+          <t>Research winches for CTD, coring and deep-tow work, 300 to 4,000 m, electric or hydraulic, with precise slow-speed control for repeatable casts.</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>A CTD cast is a measurement, not a lift</t>
+          <t>Research winches for precise, repeatable casts</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>An ROV is only as available as its umbilical winch</t>
+          <t>ROV, umbilical and personnel handling systems</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Deck machinery and handling systems for naval, coastguard and government research vessels, built to class with full material and weld traceability.</t>
+          <t>Deck machinery for naval, coastguard and government research vessels, built to class with full material and weld traceability.</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Built for government and naval programmes</t>
+          <t>Deck machinery for naval and government programmes</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">

</xml_diff>

<commit_message>
copy: equipment pages from the concise copy document
Batch 3 of the copy replacement. E-00 to E-12 rewritten as a one-line
intro and short feature lists; the Product template sets the lists in two
columns, drops the separate datasheet section (each table's footnote and
the sticky bar already carry it) and closes on the hero's two buttons and
the standard band. E-08, E-09, E-11 and E-12 leave draft.

A hub can now reword a child's row through its own cards, so the
Equipment and Winches hubs carry the document's range figures.

Spec tables are unchanged except the two figures the document marks for
checking (E-06 dry weight with level wind, E-10 15 Te parking brake),
which become RTG-to-supply markers.

Titles, descriptions and h1s updated in the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WYL1dwTrpuG7Wg2RUY2FW
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -1571,7 +1571,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>The RTG equipment range: winches, launch and recovery systems, cranes, handling systems, power units and containerised spreads for survey and subsea work.</t>
+          <t>The RTG range: winches, launch and recovery systems, cranes, tensioners, power units and containerised spreads for survey and subsea work.</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>The equipment range</t>
+          <t>Equipment range</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Marine Winches | Survey, Geotechnical &amp; ROV | RTG</t>
+          <t>Marine Winches | Survey, Geotechnical, Seismic &amp; ROV | RTG</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Electric and hydraulic marine winches from 0.3 to 7.4 tonnes working load and 200 to 5,500 m capacity, with Lebus grooved drums and controlled level wind.</t>
+          <t>Electric and hydraulic marine winches from 240 kg to 30 t WLL and up to 3,500 m capacity, with Lebus grooved drums and controlled level wind.</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Winches</t>
+          <t>Marine winches, 240 kg to 30 t WLL</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Winches for piston, gravity and box coring and CPT deployment, with constant tension control to protect the umbilical when the tool is captive in the seabed.</t>
+          <t>Winches for piston, gravity and box coring and CPT deployment, with constant tension control to protect the umbilical.</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Survey &amp; Oceanographic Winches | 300-4,000 m | RTG</t>
+          <t>Survey &amp; Oceanographic Winches | 300 to 4,000 m | RTG</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Survey and oceanographic winches in electric or hydraulic drive, with or without level wind, supplied with cable capacities from 300 to 4,000 metres.</t>
+          <t>Survey and oceanographic winches in electric or hydraulic drive, with or without level wind, with cable capacities from 300 to 4,000 metres.</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Seismic winches and source handling equipment engineered for continuous duty, high line speeds and repeated deployment cycles in marine acquisition.</t>
+          <t>Seismic winches and source handling equipment for continuous duty, high line speeds and repeated deployment cycles in marine acquisition.</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ROV, Tow &amp; Umbilical Winches | Slip Ring Ready | RTG</t>
+          <t>ROV, Tow &amp; Umbilical Winches | RTG</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>ROV, deep tow and umbilical winches with Lebus grooved drums, controlled level wind and a slip ring interface to suit your own data and power architecture.</t>
+          <t>ROV, deep-tow and umbilical winches with Lebus grooved drums, controlled level wind and a slip ring interface to suit your data and power architecture.</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Mooring, capstan and general utility winches for offshore and research vessels, built to class with the same welding and test discipline as the survey range.</t>
+          <t>Mooring, towing and utility winches for offshore and research vessels, built to class with full weld traceability and proof load testing.</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Stern and side A-frames, mini survey LARS, ROV and CTD launch and recovery systems, engineered around your deck arrangement and sea state requirement.</t>
+          <t>Stern and side A-frames, ROV and CTD launch and recovery systems, 20 to 40 Te WLL, rated to 3.9 m significant wave height.</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Launch and recovery systems</t>
+          <t>A-frames and LARS rated to 3.9 m Hs</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Deck cranes, knuckle boom and telescopic lifting equipment for research and offshore vessels, class certified and proof tested before dispatch.</t>
+          <t>Knuckle boom, telescopic and utility deck cranes, davits and personnel-rated lifting for research and offshore vessels, class certified and proof tested.</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Cranes and lifting equipment</t>
+          <t>Deck cranes and lifting equipment</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Complete handling systems for corers, seismic sources, diver baskets and subsea cable, supplied as integrated deck spreads rather than individual machines.</t>
+          <t>Complete handling systems for corers, seismic sources, diver baskets and subsea cable, supplied as integrated deck spreads.</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Self-contained two-track electro-hydraulic tensioners from 5 to 20 tonnes on a common skid, remote console controlled, for cable and pipe laying operations.</t>
+          <t>Self-contained two-track electro-hydraulic tensioners from 5 to 20 tonnes on a common skid, remote console controlled, for cable and pipe lay.</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Cable and pipe tensioners</t>
+          <t>Two-track tensioners, 5 to 20 Te</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Hydraulic power units for deck machinery, built and flushed to a defined cleanliness class and function tested with the equipment they will drive.</t>
+          <t>Hydraulic power units for deck machinery, flushed to a defined cleanliness class and function tested with the equipment they drive.</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Self-contained, road transportable handling spreads with certified lifting lugs, fork pockets and twist-lock footprints, for vessels you do not own.</t>
+          <t>Self-contained, road-transportable handling spreads with certified lifting lugs, fork pockets and twist-lock footprints for chartered vessels.</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Built to move between hulls</t>
+          <t>Portable and containerised spreads</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">

</xml_diff>

<commit_message>
copy: lifecycle pages from the concise copy document
Batch 4 of the copy replacement. L-00 to L-05 rewritten. The refurbishment
process and the six decision factors are now structured steps; the Service
template runs its steps before its body, and the Guide template lists the
factors plainly instead of pinning one to a screen. Both close on the
hero's buttons and the standard band. L-03, L-04 and L-05 leave draft, and
L-05 gets its form fields (still no backend).

Titles, descriptions and h1s updated in the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WYL1dwTrpuG7Wg2RUY2FW
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -2949,7 +2949,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Your vessel is worth more working than replaced. Condition assessment, refurbishment, capability upgrade, re-certification and spares for deck machinery.</t>
+          <t>Condition assessment, refurbishment, upgrade, re-certification and spares for deck machinery, including equipment from other manufacturers.</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Keeping equipment working</t>
+          <t>Supported for the full service life</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -3055,7 +3055,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Full refurbishment of winches, LARS and deck machinery: condition assessment, rework, component reuse, capability upgrade, testing and reissued documentation.</t>
+          <t>Refurbishment of winches, LARS and deck machinery: condition assessment, component reuse, capability upgrade, load testing and reissued documentation.</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Six questions that decide whether deck machinery is worth rebuilding: drum and shaft condition, brakes, hydraulics, capability target, spares and class status.</t>
+          <t>Six factors that decide whether deck machinery is worth rebuilding: drum and shaft, brakes, hydraulics, capability, spares and class status.</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Refurbish, upgrade or replace?</t>
+          <t>Refurbish, upgrade or replace: six factors</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Load testing, inspection and documentation for class renewal on deck machinery, including equipment originally supplied by other manufacturers.</t>
+          <t>Load testing, inspection and documentation for class renewal on deck machinery, including equipment supplied by other manufacturers.</t>
         </is>
       </c>
       <c r="L27" t="n">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Spares, technical support and field service for RTG equipment and for deck machinery supplied by others, through UK and EU offices and agents worldwide.</t>
+          <t>Spares, technical support and field service for RTG equipment and deck machinery from other manufacturers, through UK and EU offices and agents worldwide.</t>
         </is>
       </c>
       <c r="L28" t="n">
@@ -3479,7 +3479,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Tell us the equipment, the vessel and the maintenance window. We will tell you what is worth rebuilding, what is not, and what the work would involve.</t>
+          <t>Book a condition assessment for winches, LARS and deck machinery. Written report with reuse, rework and replace recommendations and costed options.</t>
         </is>
       </c>
       <c r="L29" t="n">

</xml_diff>

<commit_message>
copy: contract manufacturing pages from the concise copy document
Batch 5 of the copy replacement. C-00 to C-04 and C-06 to C-08 rewritten.
The hub lists the four tiers as linked rows with their scope, replacing
the picture carousel and the reference grid that repeated it, then sets
Approvals, IP protection, EU manufacture and Getting started in two
columns. The four tier pages share one shape: scope, two lists side by
side, one button. Ladder, Tier, Policy and Article close on the hero's
buttons and the standard band. C-08 gets its form fields (no backend).

Titles, descriptions and h1s updated in the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WYL1dwTrpuG7Wg2RUY2FW
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -3585,7 +3585,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Your design, your IP, our factory. From welded structures to complete machines, assembled, piped, wired, programmed, load tested under class and commissioned.</t>
+          <t>Your design, your IP, our factory. Structural fabrication to complete machines: assembled, piped, wired, programmed, load tested under class and commissioned.</t>
         </is>
       </c>
       <c r="L30" t="n">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>How much of your machine would you like us to take?</t>
+          <t>Contract manufacturing</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Welded structures to your drawings with EN ISO 3834 discipline, coded welders, NDT to ISO 9712 level 2 and 100 percent traceability on structural welds.</t>
+          <t>Welded structures to your drawings with EN ISO 3834 discipline, coded welders, NDT to ISO 9712 level 2 and 100% traceability on structural welds.</t>
         </is>
       </c>
       <c r="L31" t="n">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Drums, shafts, bearings, gearboxes, brakes, sheaves and level wind assembled to your specification, torqued, aligned and rotation checked before dispatch.</t>
+          <t>Drums, shafts, bearings, gearboxes, brakes, sheaves and level wind assembled to your specification, torqued, aligned and rotation checked.</t>
         </is>
       </c>
       <c r="L32" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Power units, pipework flushed to a defined cleanliness class, valve blocks, control panels, cabling, terminations and instrumentation, built to your schematics.</t>
+          <t>Power units, pipework flushed to a defined cleanliness class, valve blocks, control panels, cabling and instrumentation, built to your schematics.</t>
         </is>
       </c>
       <c r="L33" t="n">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>PLC and HMI loading, interlock proving, load testing to 150 tonnes under class witness, full certification dossier and commissioning on the vessel.</t>
+          <t>PLC and HMI loading, interlock proving, load testing to 150 tonnes under class witness, full certification dossier and vessel commissioning.</t>
         </is>
       </c>
       <c r="L34" t="n">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>NDA before drawings, segregated project files, no derivative products from client designs, and a clear contractual separation from our own equipment range.</t>
+          <t>NDA before drawings, segregated project files, no derivative products from client designs, and contractual separation from our own equipment range.</t>
         </is>
       </c>
       <c r="L36" t="n">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Your design stays yours</t>
+          <t>Design and IP protection</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Fabrication inside the EU, with melt-and-pour origin documentation supplied alongside our standard weld traceability pack for every structure we build.</t>
+          <t>Fabrication inside the EU, with melt-and-pour origin documentation supplied with our standard weld traceability pack.</t>
         </is>
       </c>
       <c r="L37" t="n">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Fabricated inside the EU, documented</t>
+          <t>EU-origin fabrication</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>A quarterly statement of available fabrication, assembly, hydraulic build and test capacity by tier, with indicative lead times for each. Updated every quarter.</t>
+          <t>Quarterly statement of available fabrication, assembly, hydraulic build and test capacity by tier, with indicative lead times.</t>
         </is>
       </c>
       <c r="L38" t="n">

</xml_diff>

<commit_message>
copy: shipyard pages from the concise copy document
Batch 6 of the copy replacement. Y-00 to Y-02 are built from empty stubs
and leave draft; Y-03 is reduced to its certifications table. The Proof
template moves the standard band to the page ending and closes on the
hero's buttons, like the other templates. Y-03's table footnote was an
internal note citing the project guide; it now says what a reader needs.

Titles, descriptions and h1s updated in the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WYL1dwTrpuG7Wg2RUY2FW
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -4637,7 +4637,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Subcontract Fabrication &amp; Deck Packages for Yards | RTG</t>
+          <t>Subcontract Fabrication &amp; Deck Packages for Shipyards | RTG</t>
         </is>
       </c>
       <c r="J40" t="n">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>European standards, EU capacity, class certified. Overflow structural fabrication and deck equipment packages that protect your delivery date.</t>
+          <t>EU capacity, class certified. Overflow structural fabrication and complete deck-equipment packages delivered to your build programme.</t>
         </is>
       </c>
       <c r="L40" t="n">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Capacity that protects your delivery date</t>
+          <t>Class-certified capacity for shipyard programmes</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4857,7 +4857,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Complete deck handling packages specified, built, tested and commissioned for newbuild survey, research and offshore vessels, integrated with your programme.</t>
+          <t>Complete deck handling packages engineered, built, tested and commissioned for newbuild survey, research and offshore vessels.</t>
         </is>
       </c>
       <c r="L42" t="n">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Deck equipment packages</t>
+          <t>Deck-equipment packages for newbuilds</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Bureau Veritas Mode II recognition, welding procedures approved with TUV, DNV and Lloyd's Register, welders to ISO 9606-1 and NDT to ISO 9712 level 2.</t>
+          <t>Bureau Veritas Mode II recognition, welding procedures approved with TÜV, DNV and Lloyd's Register, welders to ISO 9606-1 and NDT to ISO 9712 level 2.</t>
         </is>
       </c>
       <c r="L43" t="n">

</xml_diff>

<commit_message>
copy: proof pages from the concise copy document
Batch 7 of the copy replacement. P-00, P-01, P-03, P-06, P-07 and P-08
rewritten. P-01, P-07 and P-08 are built from empty stubs and leave draft.
The test facility and case study pages become a short table and a few
lines each; the Case template closes on the hero's buttons and the
standard band. Client names are published as written in the document.

Titles, descriptions and h1s updated in the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WYL1dwTrpuG7Wg2RUY2FW
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -5175,7 +5175,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Twenty-two years, more than 250 completed projects and around 1,500 deck machines. Case studies, vessel references, our test facility and what clients say.</t>
+          <t>Family business since 1978: more than 250 completed projects and around 1,500 deck machines. Case studies, references and our test facility.</t>
         </is>
       </c>
       <c r="L45" t="n">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>The evidence</t>
+          <t>Track record</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -5281,7 +5281,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>How RTG standardised handling across a survey fleet, rebuilt a twelve-year-old traction winch, and built complete machines to an OEM's drawings.</t>
+          <t>Fleet standardisation across seven Fugro vessels, a rebuilt 2009 traction winch, contract manufacturing and a shipyard newbuild programme.</t>
         </is>
       </c>
       <c r="L46" t="n">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>A twelve-year-old electro-hydraulic traction winch assessed, rebuilt, upgraded and retested for offshore geotechnical work, with documentation reissued.</t>
+          <t>A 2009 electro-hydraulic traction winch assessed, rebuilt, upgraded and retested for offshore geotechnical work, with documentation reissued.</t>
         </is>
       </c>
       <c r="L48" t="n">
@@ -5501,7 +5501,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>The winch we built in 2009, rebuilt in 2021</t>
+          <t>2009 traction winch, rebuilt in 2021</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Two test stands, load testing to 150 tonnes with certified weights: proof load, dynamic functional, brake holding, render and speed tests under class witness.</t>
+          <t>Two test stands, load testing to 150 tonnes with certified weights: proof load, dynamic, brake holding, render and speed tests under class witness.</t>
         </is>
       </c>
       <c r="L51" t="n">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Nothing leaves this factory untested</t>
+          <t>Test facility: two stands, 150 Te</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -5917,7 +5917,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>More than 50 global customers and research institutions, over 250 completed projects and around 1,500 custom deck machines delivered since 2003.</t>
+          <t>More than 50 operators, OEMs, shipyards and research institutions; over 250 projects and around 1,500 custom deck machines since 1978.</t>
         </is>
       </c>
       <c r="L52" t="n">
@@ -5925,7 +5925,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Vessels and clients</t>
+          <t>Clients</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>In the words of a global survey operator, a major shipyard and an offshore equipment specialist, on design quality, communication and on-time delivery.</t>
+          <t>Operators, shipyards and equipment manufacturers on RTG's design quality, communication and on-time delivery.</t>
         </is>
       </c>
       <c r="L53" t="n">

</xml_diff>

<commit_message>
copy: about and contact pages from the concise copy document
Batch 8, the last of the copy replacement. A-01 rewritten; A-02, A-05,
X-01, X-02 and X-03 built from stubs and leave draft. The contact page
publishes the two office addresses and takes its enquiry routes from its
own cards; X-03 gets its form fields (no backend). About, Careers and
Contact close on the hero's buttons and the standard band.

CLAUDE.md: the September intake table is retired and the About and
Contact template notes brought up to date.

Titles, descriptions and h1s updated in the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WYL1dwTrpuG7Wg2RUY2FW
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -6545,7 +6545,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>About RTG | British Design, European Manufacture</t>
+          <t>About RTG | Family Business in Deck Machinery Since 1978</t>
         </is>
       </c>
       <c r="J58" t="n">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Founded to combine British deck equipment design with European manufacturing. Twenty-two years, 250 projects and around 1,500 machines delivered.</t>
+          <t>Family-owned since 1978. British deck machinery design and European manufacturing: 1,500 machines and 250 projects for 50+ clients.</t>
         </is>
       </c>
       <c r="L58" t="n">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>A father, a son, and a factory in Satu Mare</t>
+          <t>A family business in deck machinery since 1978</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -6659,7 +6659,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Around 80 engineers, welders, fitters and technicians in a purpose-built facility in Satu Mare, Romania, with design and commercial teams in the UK.</t>
+          <t>Around 80 engineers, welders, fitters and technicians in Satu Mare, Romania, with design and commercial teams in the UK.</t>
         </is>
       </c>
       <c r="L59" t="n">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>The people and the place</t>
+          <t>People and facility</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -6977,7 +6977,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Welding, mechanical, hydraulic, electrical, automation and design roles in Satu Mare and the UK. See what we build and who you would build it with.</t>
+          <t>Welding, mechanical, hydraulic, electrical, automation and design roles in Satu Mare and the UK.</t>
         </is>
       </c>
       <c r="L62" t="n">
@@ -6985,7 +6985,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>Build things that go to sea</t>
+          <t>Careers</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Talk to our UK commercial team or our factory at Satu Mare in Romania, or find your regional agent across the Americas and Asia Pacific. We answer quickly.</t>
+          <t>Contact our UK commercial team or our Satu Mare factory, or find your regional agent in the Americas and Asia Pacific.</t>
         </is>
       </c>
       <c r="L63" t="n">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Contact us</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -7181,7 +7181,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Our Agents in the Americas and Asia Pacific | RTG</t>
+          <t>RTG Agents in the Americas and Asia Pacific | RTG</t>
         </is>
       </c>
       <c r="J64" t="n">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Local representation for sales, support and spares across the Americas and Asia Pacific, backed directly by the engineers who designed and built the equipment.</t>
+          <t>Local sales, support and spares in the Americas and Asia Pacific, backed by the engineers who designed and built the equipment.</t>
         </is>
       </c>
       <c r="L64" t="n">
@@ -7197,7 +7197,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Where to find us</t>
+          <t>Agents</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Tell us the duty, the vessel and the timescale. We will come back with a proposed configuration and an indicative price, and say what we still need.</t>
+          <t>Send the duty, vessel and timescale for a proposed configuration and indicative price.</t>
         </is>
       </c>
       <c r="L65" t="n">

</xml_diff>

<commit_message>
equipment: finder on the hub, from the datasheet index
Search and filter 91 standard designs on /equipment/ by type,
application, drive, working load and cable capacity. Data is
generated by scripts/build-equipment.mjs from RTG's datasheet index
workbook, reading a whitelist of publishable columns; the workbook
itself is gitignored. Rows whose description and figures disagree are
left out and reported.

Headline ranges follow the datasheets: winches 240 kg to 48 t,
A-frames 5 to 40 Te.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015WYL1dwTrpuG7Wg2RUY2FW
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -1677,7 +1677,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Electric and hydraulic marine winches from 240 kg to 30 t WLL and up to 3,500 m capacity, with Lebus grooved drums and controlled level wind.</t>
+          <t>Electric and hydraulic marine winches from 240 kg to 48 t WLL and up to 3,500 m capacity, with Lebus grooved drums and controlled level wind.</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Marine winches, 240 kg to 30 t WLL</t>
+          <t>Marine winches, 240 kg to 48 t WLL</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Stern and side A-frames, ROV and CTD launch and recovery systems, 20 to 40 Te WLL, rated to 3.9 m significant wave height.</t>
+          <t>Stern and side A-frames, ROV and CTD launch and recovery systems, 5 to 40 Te WLL, rated to 3.9 m significant wave height.</t>
         </is>
       </c>
       <c r="L18" t="n">

</xml_diff>